<commit_message>
docs: align project brief and roadmap on Airflow and Docker
The orchestrator and container runtime were settled (Apache Airflow,
Docker) but the project brief still read "Prefect (ou Airflow)" and the
roadmaps still mentioned Prefect and Podman.

Updated the brief, the monthly checkpoints roadmap and both roadmap
spreadsheets. roadmap.png is an image and was not regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Roadmap/roadmap_churn_2026-2027.xlsx
+++ b/Roadmap/roadmap_churn_2026-2027.xlsx
@@ -968,7 +968,7 @@
       <c r="A13" s="16" t="n"/>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>Pipeline ingestion Bronze→Silver (dbt · Prefect)</t>
+          <t>Pipeline ingestion Bronze→Silver (dbt · Airflow)</t>
         </is>
       </c>
       <c r="C13" s="19" t="n"/>
@@ -1156,7 +1156,7 @@
       <c r="A21" s="16" t="n"/>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>Conteneurisation Podman + docker-compose</t>
+          <t>Conteneurisation Docker + docker-compose</t>
         </is>
       </c>
       <c r="C21" s="19" t="n"/>

</xml_diff>